<commit_message>
11. GameWindow UI Scale Fixed, Inventory Manager Add
GameWindow Scene의 UI 비율 조정.
InventoryManager의 추가로 ItemSystem 일부 구현.
</commit_message>
<xml_diff>
--- a/Assets/Resources/StatusData.xlsx
+++ b/Assets/Resources/StatusData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monke\Desktop\war_LIke2\Assets\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47A25B83-0E68-43C9-9EF8-578491DF0C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC739E6B-13FE-4822-82DB-5607A16CF55F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{C74F93A7-7243-4DE6-AFA9-670647F89833}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="28">
   <si>
     <t>StatusData</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -124,6 +124,18 @@
   </si>
   <si>
     <t>선</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>악</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_005</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>더미봇</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -771,16 +783,36 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.6">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
+      <c r="A9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="1">
+        <v>10</v>
+      </c>
+      <c r="E9" s="1">
+        <v>10</v>
+      </c>
+      <c r="F9" s="1">
+        <v>10</v>
+      </c>
+      <c r="G9" s="1">
+        <v>10</v>
+      </c>
+      <c r="H9" s="1">
+        <v>10</v>
+      </c>
+      <c r="I9" s="1">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.6">
       <c r="A10" s="1"/>

</xml_diff>